<commit_message>
svm fixes, add configs
</commit_message>
<xml_diff>
--- a/baselines/svm-baseline/detected_events.xlsx
+++ b/baselines/svm-baseline/detected_events.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C26"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -435,10 +435,10 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>5.5</v>
+        <v>61.05</v>
       </c>
       <c r="B2" t="n">
-        <v>46</v>
+        <v>67.55</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -448,49 +448,49 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>48.5</v>
+        <v>78.55</v>
       </c>
       <c r="B3" t="n">
-        <v>55</v>
+        <v>125.05</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>eID_2</t>
+          <t>eID_5</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>60</v>
+        <v>129.05</v>
       </c>
       <c r="B4" t="n">
-        <v>114.5</v>
+        <v>131.55</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>eID_5</t>
+          <t>eID_1</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>117.5</v>
+        <v>152.55</v>
       </c>
       <c r="B5" t="n">
-        <v>118.5</v>
+        <v>158.05</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>eID_1</t>
+          <t>eID_2</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>122</v>
+        <v>170.55</v>
       </c>
       <c r="B6" t="n">
-        <v>123.5</v>
+        <v>172.55</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -500,261 +500,53 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>128.5</v>
+        <v>182.55</v>
       </c>
       <c r="B7" t="n">
-        <v>128.5</v>
+        <v>183.55</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>eID_2</t>
+          <t>eID_1</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>129</v>
+        <v>195.55</v>
       </c>
       <c r="B8" t="n">
-        <v>131.5</v>
+        <v>200.55</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>eID_1</t>
+          <t>eID_5</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>134.5</v>
+        <v>214.55</v>
       </c>
       <c r="B9" t="n">
-        <v>145.5</v>
+        <v>215.05</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>eID_5</t>
+          <t>eID_1</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>147.5</v>
+        <v>226.55</v>
       </c>
       <c r="B10" t="n">
-        <v>147.5</v>
+        <v>247.05</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>eID_1</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="n">
-        <v>152</v>
-      </c>
-      <c r="B11" t="n">
-        <v>158</v>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>eID_2</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="n">
-        <v>170.5</v>
-      </c>
-      <c r="B12" t="n">
-        <v>172.5</v>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
           <t>eID_5</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="n">
-        <v>181</v>
-      </c>
-      <c r="B13" t="n">
-        <v>181</v>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>eID_2</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="n">
-        <v>183</v>
-      </c>
-      <c r="B14" t="n">
-        <v>183.5</v>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>eID_1</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="n">
-        <v>185.5</v>
-      </c>
-      <c r="B15" t="n">
-        <v>205.5</v>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>eID_5</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="n">
-        <v>208</v>
-      </c>
-      <c r="B16" t="n">
-        <v>208</v>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>eID_2</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="n">
-        <v>212.5</v>
-      </c>
-      <c r="B17" t="n">
-        <v>215.5</v>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>eID_1</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="n">
-        <v>219</v>
-      </c>
-      <c r="B18" t="n">
-        <v>246.5</v>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>eID_5</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="n">
-        <v>247</v>
-      </c>
-      <c r="B19" t="n">
-        <v>248.5</v>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>eID_4</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="n">
-        <v>251</v>
-      </c>
-      <c r="B20" t="n">
-        <v>252</v>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>eID_2</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="n">
-        <v>252.5</v>
-      </c>
-      <c r="B21" t="n">
-        <v>254.5</v>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>eID_5</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="n">
-        <v>257</v>
-      </c>
-      <c r="B22" t="n">
-        <v>257.5</v>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>eID_2</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="n">
-        <v>264</v>
-      </c>
-      <c r="B23" t="n">
-        <v>271.5</v>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>eID_1</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="n">
-        <v>273.5</v>
-      </c>
-      <c r="B24" t="n">
-        <v>273.5</v>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>eID_5</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="n">
-        <v>275</v>
-      </c>
-      <c r="B25" t="n">
-        <v>285.5</v>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>eID_2</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="n">
-        <v>294.5</v>
-      </c>
-      <c r="B26" t="n">
-        <v>299.5</v>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>eID_1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
train model on public database
</commit_message>
<xml_diff>
--- a/baselines/svm-baseline/detected_events.xlsx
+++ b/baselines/svm-baseline/detected_events.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -435,118 +435,222 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>61.05</v>
+        <v>1432.519</v>
       </c>
       <c r="B2" t="n">
-        <v>67.55</v>
+        <v>1440.019</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>eID_5</t>
+          <t>413.0</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>78.55</v>
+        <v>1451.019</v>
       </c>
       <c r="B3" t="n">
-        <v>125.05</v>
+        <v>1452.019</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>eID_5</t>
+          <t>413.0</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>129.05</v>
+        <v>1457.019</v>
       </c>
       <c r="B4" t="n">
-        <v>131.55</v>
+        <v>1463.519</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>eID_1</t>
+          <t>413.0</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>152.55</v>
+        <v>1467.519</v>
       </c>
       <c r="B5" t="n">
-        <v>158.05</v>
+        <v>1474.519</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>eID_2</t>
+          <t>412.0</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>170.55</v>
+        <v>1481.019</v>
       </c>
       <c r="B6" t="n">
-        <v>172.55</v>
+        <v>1490.519</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>eID_5</t>
+          <t>413.0</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>182.55</v>
+        <v>1496.019</v>
       </c>
       <c r="B7" t="n">
-        <v>183.55</v>
+        <v>1496.519</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>eID_1</t>
+          <t>406.0</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>195.55</v>
+        <v>1499.519</v>
       </c>
       <c r="B8" t="n">
-        <v>200.55</v>
+        <v>1500.019</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>eID_5</t>
+          <t>413.0</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>214.55</v>
+        <v>1512.519</v>
       </c>
       <c r="B9" t="n">
-        <v>215.05</v>
+        <v>1513.019</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>eID_1</t>
+          <t>413.0</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>226.55</v>
+        <v>1518.019</v>
       </c>
       <c r="B10" t="n">
-        <v>247.05</v>
+        <v>1539.519</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>eID_5</t>
+          <t>405.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>1541.019</v>
+      </c>
+      <c r="B11" t="n">
+        <v>1542.019</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>412.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>1542.519</v>
+      </c>
+      <c r="B12" t="n">
+        <v>1544.019</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>413.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>1554.519</v>
+      </c>
+      <c r="B13" t="n">
+        <v>1567.019</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>405.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>1569.019</v>
+      </c>
+      <c r="B14" t="n">
+        <v>1570.019</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>406.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>1574.519</v>
+      </c>
+      <c r="B15" t="n">
+        <v>1575.019</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>405.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>1584.019</v>
+      </c>
+      <c r="B16" t="n">
+        <v>1589.019</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>404.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>1630.019</v>
+      </c>
+      <c r="B17" t="n">
+        <v>1631.019</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>413.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>1657.519</v>
+      </c>
+      <c r="B18" t="n">
+        <v>1658.519</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>413.0</t>
         </is>
       </c>
     </row>

</xml_diff>